<commit_message>
fix: add fake GROQ_API_KEY to phpunit.xml so Http::fake() works in CI
Admin role management tests: 6/6 passed
Total test suite: 84 passed (272 assertions)
</commit_message>
<xml_diff>
--- a/artefacts/backlog/product_backlog_full.xlsx
+++ b/artefacts/backlog/product_backlog_full.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hiba9\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hiba9\safe-stay-ai\artefacts\backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D25FC08-E651-45F5-A1CD-CC5221B3CC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C67A9E-719F-4935-8A69-0325C4E69C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="212">
   <si>
     <t>SWE6011 Agile Programming · Assignment 2 · Numair Alsaleh (2529226)</t>
   </si>
@@ -150,9 +150,6 @@
   </si>
   <si>
     <t>9 Apr</t>
-  </si>
-  <si>
-    <t>View all users; change roles; deactivate accounts; changes instant; actions logged</t>
   </si>
   <si>
     <t>T2</t>
@@ -719,6 +716,9 @@
   </si>
   <si>
     <t xml:space="preserve">Safe-Stay AI - Product Backlog </t>
+  </si>
+  <si>
+    <t>View all users; change roles; changes instant; actions logged</t>
   </si>
 </sst>
 </file>
@@ -1125,16 +1125,6 @@
     <xf numFmtId="0" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1165,16 +1155,26 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1494,31 +1494,31 @@
   <sheetData>
     <row r="1" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="71" t="s">
-        <v>211</v>
-      </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
+        <v>210</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
     </row>
     <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
     </row>
     <row r="3" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1543,13 +1543,13 @@
         <v>7</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="68" t="s">
-        <v>206</v>
+      <c r="J3" s="64" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
@@ -1562,8 +1562,8 @@
       <c r="C4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="64" t="s">
-        <v>194</v>
+      <c r="D4" s="60" t="s">
+        <v>193</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>11</v>
@@ -1571,8 +1571,8 @@
       <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="72" t="s">
-        <v>144</v>
+      <c r="G4" s="67" t="s">
+        <v>143</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>15</v>
@@ -1707,21 +1707,21 @@
         <v>36</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>37</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>38</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>39</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>20</v>
@@ -1729,31 +1729,31 @@
       <c r="F9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="70" t="s">
-        <v>74</v>
+      <c r="G9" s="66" t="s">
+        <v>73</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="J9" s="69" t="s">
-        <v>198</v>
+      <c r="J9" s="65" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>20</v>
@@ -1768,24 +1768,24 @@
         <v>26</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="J10" s="69" t="s">
-        <v>199</v>
+        <v>44</v>
+      </c>
+      <c r="J10" s="65" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>20</v>
@@ -1797,27 +1797,27 @@
         <v>14</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="J11" s="69" t="s">
-        <v>200</v>
+        <v>44</v>
+      </c>
+      <c r="J11" s="65" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>20</v>
@@ -1832,24 +1832,24 @@
         <v>26</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J12" s="69" t="s">
-        <v>201</v>
+        <v>49</v>
+      </c>
+      <c r="J12" s="65" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>29</v>
@@ -1861,18 +1861,18 @@
         <v>14</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="J13" s="69" t="s">
-        <v>202</v>
+        <v>52</v>
+      </c>
+      <c r="J13" s="65" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>10</v>
@@ -1880,8 +1880,8 @@
       <c r="C14" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="65" t="s">
-        <v>195</v>
+      <c r="D14" s="61" t="s">
+        <v>194</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>11</v>
@@ -1889,8 +1889,8 @@
       <c r="F14" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="73" t="s">
-        <v>144</v>
+      <c r="G14" s="68" t="s">
+        <v>143</v>
       </c>
       <c r="H14" s="11" t="s">
         <v>15</v>
@@ -1902,16 +1902,16 @@
     </row>
     <row r="15" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>20</v>
@@ -1926,24 +1926,24 @@
         <v>21</v>
       </c>
       <c r="I15" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J15" s="16" t="s">
         <v>58</v>
-      </c>
-      <c r="J15" s="16" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>20</v>
@@ -1958,24 +1958,24 @@
         <v>21</v>
       </c>
       <c r="I16" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="J16" s="16" t="s">
         <v>62</v>
-      </c>
-      <c r="J16" s="16" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>29</v>
@@ -1990,24 +1990,24 @@
         <v>26</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>29</v>
@@ -2022,24 +2022,24 @@
         <v>26</v>
       </c>
       <c r="I18" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="J18" s="16" t="s">
         <v>69</v>
-      </c>
-      <c r="J18" s="16" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>72</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>20</v>
@@ -2048,30 +2048,30 @@
         <v>13</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H19" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I19" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="J19" s="69" t="s">
-        <v>203</v>
+      <c r="J19" s="65" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>76</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>20</v>
@@ -2086,24 +2086,24 @@
         <v>26</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J20" s="69" t="s">
-        <v>204</v>
+        <v>49</v>
+      </c>
+      <c r="J20" s="65" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>78</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>20</v>
@@ -2118,15 +2118,15 @@
         <v>26</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="J21" s="69" t="s">
-        <v>205</v>
+        <v>78</v>
+      </c>
+      <c r="J21" s="65" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>10</v>
@@ -2134,44 +2134,44 @@
       <c r="C22" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="66" t="s">
-        <v>196</v>
+      <c r="D22" s="62" t="s">
+        <v>195</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G22" s="17" t="s">
         <v>14</v>
       </c>
       <c r="H22" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="I22" s="17" t="s">
         <v>83</v>
-      </c>
-      <c r="I22" s="17" t="s">
-        <v>84</v>
       </c>
       <c r="J22" s="22"/>
     </row>
     <row r="23" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>18</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E23" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G23" s="20" t="s">
         <v>14</v>
@@ -2180,62 +2180,62 @@
         <v>21</v>
       </c>
       <c r="I23" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="J23" s="22" t="s">
         <v>87</v>
-      </c>
-      <c r="J23" s="22" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>18</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E24" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F24" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G24" s="20" t="s">
         <v>14</v>
       </c>
       <c r="H24" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="I24" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="I24" s="20" t="s">
+      <c r="J24" s="22" t="s">
         <v>92</v>
-      </c>
-      <c r="J24" s="22" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E25" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F25" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G25" s="20" t="s">
         <v>14</v>
@@ -2244,30 +2244,30 @@
         <v>21</v>
       </c>
       <c r="I25" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="J25" s="22" t="s">
         <v>96</v>
-      </c>
-      <c r="J25" s="22" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B26" s="21" t="s">
         <v>18</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E26" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F26" s="20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G26" s="20" t="s">
         <v>14</v>
@@ -2276,79 +2276,79 @@
         <v>26</v>
       </c>
       <c r="I26" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="J26" s="22" t="s">
         <v>100</v>
-      </c>
-      <c r="J26" s="22" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>102</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C27" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>103</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>20</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>14</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="J27" s="69" t="s">
-        <v>207</v>
+        <v>103</v>
+      </c>
+      <c r="J27" s="65" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C28" s="10" t="s">
+      <c r="E28" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>82</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>14</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="J28" s="69" t="s">
-        <v>208</v>
+        <v>106</v>
+      </c>
+      <c r="J28" s="65" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="24" t="s">
         <v>10</v>
@@ -2356,44 +2356,44 @@
       <c r="C29" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="67" t="s">
-        <v>197</v>
+      <c r="D29" s="63" t="s">
+        <v>196</v>
       </c>
       <c r="E29" s="23" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G29" s="23" t="s">
         <v>14</v>
       </c>
       <c r="H29" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="I29" s="23" t="s">
         <v>111</v>
-      </c>
-      <c r="I29" s="23" t="s">
-        <v>112</v>
       </c>
       <c r="J29" s="25"/>
     </row>
     <row r="30" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" s="27" t="s">
         <v>18</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E30" s="26" t="s">
         <v>20</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G30" s="26" t="s">
         <v>14</v>
@@ -2402,30 +2402,30 @@
         <v>21</v>
       </c>
       <c r="I30" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J30" s="28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B31" s="27" t="s">
         <v>18</v>
       </c>
       <c r="C31" s="28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E31" s="26" t="s">
         <v>20</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G31" s="26" t="s">
         <v>14</v>
@@ -2434,30 +2434,30 @@
         <v>26</v>
       </c>
       <c r="I31" s="26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J31" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B32" s="27" t="s">
         <v>18</v>
       </c>
       <c r="C32" s="28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D32" s="28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E32" s="26" t="s">
         <v>29</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G32" s="26" t="s">
         <v>14</v>
@@ -2466,30 +2466,30 @@
         <v>26</v>
       </c>
       <c r="I32" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="J32" s="28" t="s">
         <v>121</v>
-      </c>
-      <c r="J32" s="28" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B33" s="27" t="s">
         <v>18</v>
       </c>
       <c r="C33" s="28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D33" s="28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E33" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F33" s="26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G33" s="26" t="s">
         <v>14</v>
@@ -2498,106 +2498,106 @@
         <v>26</v>
       </c>
       <c r="I33" s="26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J33" s="28" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="57" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="61" t="s">
+      <c r="B34" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="58" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="B34" s="61" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" s="62" t="s">
-        <v>109</v>
-      </c>
-      <c r="D34" s="62" t="s">
+      <c r="E34" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="57" t="s">
+        <v>14</v>
+      </c>
+      <c r="H34" s="57" t="s">
+        <v>40</v>
+      </c>
+      <c r="I34" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="E34" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" s="61" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="H34" s="61" t="s">
-        <v>41</v>
-      </c>
-      <c r="I34" s="61" t="s">
+      <c r="J34" s="65" t="s">
         <v>128</v>
       </c>
-      <c r="J34" s="69" t="s">
+    </row>
+    <row r="35" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="66" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="70" t="s">
-        <v>130</v>
-      </c>
       <c r="B35" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E35" s="8" t="s">
         <v>20</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>14</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="J35" s="69" t="s">
-        <v>209</v>
+        <v>134</v>
+      </c>
+      <c r="J35" s="65" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="70" t="s">
-        <v>133</v>
+      <c r="A36" s="66" t="s">
+        <v>132</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>20</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>14</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="J36" s="69" t="s">
-        <v>210</v>
+        <v>131</v>
+      </c>
+      <c r="J36" s="65" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -2624,30 +2624,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="58" t="s">
-        <v>136</v>
-      </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
+      <c r="A1" s="72" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
@@ -2658,39 +2658,39 @@
         <v>13</v>
       </c>
       <c r="B3" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="63" t="s">
+      <c r="D3" s="59" t="s">
+        <v>192</v>
+      </c>
+      <c r="E3" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="63" t="s">
-        <v>193</v>
-      </c>
-      <c r="E3" s="63" t="s">
+      <c r="F3" s="30" t="s">
         <v>143</v>
-      </c>
-      <c r="F3" s="30" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="32" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B4" s="33" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="69" t="s">
         <v>145</v>
       </c>
-      <c r="C4" s="74" t="s">
+      <c r="D4" s="69" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="74" t="s">
+      <c r="E4" s="69" t="s">
         <v>147</v>
       </c>
-      <c r="E4" s="74" t="s">
+      <c r="F4" s="33" t="s">
         <v>148</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2715,33 +2715,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="58" t="s">
-        <v>150</v>
-      </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
+      <c r="A1" s="72" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
@@ -2755,10 +2755,10 @@
         <v>13</v>
       </c>
       <c r="D3" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="31" t="s">
         <v>156</v>
-      </c>
-      <c r="E3" s="31" t="s">
-        <v>157</v>
       </c>
       <c r="F3" s="30">
         <f>9+7</f>
@@ -2767,19 +2767,19 @@
     </row>
     <row r="4" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>54</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>55</v>
       </c>
       <c r="C4" s="36" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="37" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" s="37" t="s">
         <v>158</v>
-      </c>
-      <c r="E4" s="37" t="s">
-        <v>159</v>
       </c>
       <c r="F4" s="36">
         <f>10+5</f>
@@ -2788,19 +2788,19 @@
     </row>
     <row r="5" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="C5" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="C5" s="33" t="s">
-        <v>82</v>
-      </c>
       <c r="D5" s="34" t="s">
+        <v>159</v>
+      </c>
+      <c r="E5" s="34" t="s">
         <v>160</v>
-      </c>
-      <c r="E5" s="34" t="s">
-        <v>161</v>
       </c>
       <c r="F5" s="33">
         <f>13+2</f>
@@ -2809,19 +2809,19 @@
     </row>
     <row r="6" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="C6" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="39" t="s">
-        <v>110</v>
-      </c>
       <c r="D6" s="40" t="s">
+        <v>161</v>
+      </c>
+      <c r="E6" s="40" t="s">
         <v>162</v>
-      </c>
-      <c r="E6" s="40" t="s">
-        <v>163</v>
       </c>
       <c r="F6" s="39">
         <f>9+3</f>
@@ -2830,7 +2830,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E7" s="41" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F7" s="41">
         <f>SUM(F3:F6)</f>
@@ -2860,38 +2860,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="58" t="s">
-        <v>165</v>
-      </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
+      <c r="A1" s="72" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>7</v>
@@ -2899,13 +2899,13 @@
     </row>
     <row r="3" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="42" t="s">
+        <v>170</v>
+      </c>
+      <c r="B3" s="43" t="s">
         <v>171</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="C3" s="44" t="s">
         <v>172</v>
-      </c>
-      <c r="C3" s="44" t="s">
-        <v>173</v>
       </c>
       <c r="D3" s="44" t="s">
         <v>29</v>
@@ -2914,24 +2914,24 @@
         <v>20</v>
       </c>
       <c r="F3" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="G3" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="H3" s="44" t="s">
         <v>175</v>
-      </c>
-      <c r="H3" s="44" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="45" t="s">
+        <v>176</v>
+      </c>
+      <c r="B4" s="46" t="s">
         <v>177</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="C4" s="47" t="s">
         <v>178</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>179</v>
       </c>
       <c r="D4" s="47" t="s">
         <v>20</v>
@@ -2940,27 +2940,27 @@
         <v>20</v>
       </c>
       <c r="F4" s="47" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G4" s="46" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H4" s="47" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="48" t="s">
+        <v>180</v>
+      </c>
+      <c r="B5" s="49" t="s">
         <v>181</v>
       </c>
-      <c r="B5" s="49" t="s">
-        <v>182</v>
-      </c>
       <c r="C5" s="50" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D5" s="50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E5" s="50" t="s">
         <v>29</v>
@@ -2969,24 +2969,24 @@
         <v>29</v>
       </c>
       <c r="G5" s="49" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H5" s="50" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="B6" s="52" t="s">
         <v>184</v>
       </c>
-      <c r="B6" s="52" t="s">
-        <v>185</v>
-      </c>
       <c r="C6" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D6" s="53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E6" s="53" t="s">
         <v>29</v>
@@ -2995,24 +2995,24 @@
         <v>29</v>
       </c>
       <c r="G6" s="52" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H6" s="53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="54" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="55" t="s">
         <v>187</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="C7" s="56" t="s">
         <v>188</v>
       </c>
-      <c r="C7" s="56" t="s">
-        <v>189</v>
-      </c>
       <c r="D7" s="56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7" s="56" t="s">
         <v>20</v>
@@ -3021,35 +3021,35 @@
         <v>20</v>
       </c>
       <c r="G7" s="55" t="s">
+        <v>189</v>
+      </c>
+      <c r="H7" s="56" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="74" t="s">
         <v>190</v>
       </c>
-      <c r="H7" s="56" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="59" t="s">
+      <c r="B8" s="73"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="73"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
+    </row>
+    <row r="9" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="74" t="s">
         <v>191</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
-    </row>
-    <row r="9" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="59" t="s">
-        <v>192</v>
-      </c>
-      <c r="B9" s="57"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="57"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
+      <c r="B9" s="73"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="73"/>
+      <c r="F9" s="73"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
chore: add Sprint 2 artefacts and fix ManualController whitespace
</commit_message>
<xml_diff>
--- a/artefacts/backlog/product_backlog_full.xlsx
+++ b/artefacts/backlog/product_backlog_full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hiba9\safe-stay-ai\artefacts\backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C67A9E-719F-4935-8A69-0325C4E69C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93C5494-D7E2-44D7-9D00-EC6A6CEF3F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="213">
   <si>
     <t>SWE6011 Agile Programming · Assignment 2 · Numair Alsaleh (2529226)</t>
   </si>
@@ -719,6 +719,9 @@
   </si>
   <si>
     <t>View all users; change roles; changes instant; actions logged</t>
+  </si>
+  <si>
+    <t>Very Low</t>
   </si>
 </sst>
 </file>
@@ -2908,7 +2911,7 @@
         <v>172</v>
       </c>
       <c r="D3" s="44" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E3" s="44" t="s">
         <v>20</v>
@@ -2934,7 +2937,7 @@
         <v>178</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="E4" s="47" t="s">
         <v>20</v>
@@ -2960,7 +2963,7 @@
         <v>172</v>
       </c>
       <c r="D5" s="50" t="s">
-        <v>70</v>
+        <v>212</v>
       </c>
       <c r="E5" s="50" t="s">
         <v>29</v>
@@ -2986,7 +2989,7 @@
         <v>172</v>
       </c>
       <c r="D6" s="53" t="s">
-        <v>70</v>
+        <v>212</v>
       </c>
       <c r="E6" s="53" t="s">
         <v>29</v>
@@ -3012,7 +3015,7 @@
         <v>188</v>
       </c>
       <c r="D7" s="56" t="s">
-        <v>70</v>
+        <v>212</v>
       </c>
       <c r="E7" s="56" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
chore: add burndown charts, Sprint 2 closing screenshots, and Zephyr test cycle evidence
</commit_message>
<xml_diff>
--- a/artefacts/backlog/product_backlog_full.xlsx
+++ b/artefacts/backlog/product_backlog_full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hiba9\safe-stay-ai\artefacts\backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93C5494-D7E2-44D7-9D00-EC6A6CEF3F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D778616-FCE0-4B1C-986C-C2CC60537626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -1605,7 +1605,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>21</v>
@@ -1637,7 +1637,7 @@
         <v>13</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
chore: update artefacts and add final report
</commit_message>
<xml_diff>
--- a/artefacts/backlog/product_backlog_full.xlsx
+++ b/artefacts/backlog/product_backlog_full.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hiba9\safe-stay-ai\artefacts\backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D778616-FCE0-4B1C-986C-C2CC60537626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B43148E-2EA9-49EB-A5B5-1C2B274E4A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Epic Summary" sheetId="3" r:id="rId3"/>
     <sheet name="Risk Log" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="210">
   <si>
     <t>SWE6011 Agile Programming · Assignment 2 · Numair Alsaleh (2529226)</t>
   </si>
@@ -83,9 +83,6 @@
     <t>Sprint 1</t>
   </si>
   <si>
-    <t>To Do</t>
-  </si>
-  <si>
     <t>19</t>
   </si>
   <si>
@@ -584,9 +581,6 @@
     <t>R3</t>
   </si>
   <si>
-    <t>OpenAI API cost or rate limits during development</t>
-  </si>
-  <si>
     <t>Use Groq free tier during development; mock API responses in PHPUnit tests; switch to real API for demo only</t>
   </si>
   <si>
@@ -609,12 +603,6 @@
   </si>
   <si>
     <t>All screenshots committed to GitHub artefacts folder immediately after capture; never rely on Jira alone</t>
-  </si>
-  <si>
-    <t>Sprint 1 Risk Review (14 April 2026) — [Complete at end of Sprint 1]</t>
-  </si>
-  <si>
-    <t>Sprint 2 Risk Review (25 April 2026) — [Complete at end of Sprint 2]</t>
   </si>
   <si>
     <t xml:space="preserve">SSAI-5,6,7,8 (Auth) · SSAI-9,10,11,12 (Property) · T1-T8, T11 (Tasks) </t>
@@ -722,6 +710,9 @@
   </si>
   <si>
     <t>Very Low</t>
+  </si>
+  <si>
+    <t>Groq API rate limits or downtime during development</t>
   </si>
 </sst>
 </file>
@@ -958,7 +949,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1179,6 +1170,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1497,7 +1497,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="71" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B1" s="72"/>
       <c r="C1" s="72"/>
@@ -1546,13 +1546,13 @@
         <v>7</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J3" s="64" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
@@ -1566,7 +1566,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="60" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>11</v>
@@ -1575,307 +1575,307 @@
         <v>13</v>
       </c>
       <c r="G4" s="67" t="s">
-        <v>143</v>
+        <v>72</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="J4" s="7"/>
     </row>
     <row r="5" spans="1:10" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>73</v>
+      <c r="G5" s="67" t="s">
+        <v>72</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="J5" s="7" t="s">
         <v>22</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>73</v>
+      <c r="G6" s="67" t="s">
+        <v>72</v>
       </c>
       <c r="H6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="J6" s="7" t="s">
         <v>27</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>14</v>
+      <c r="G7" s="67" t="s">
+        <v>72</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>32</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="45.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>14</v>
+      <c r="G8" s="67" t="s">
+        <v>72</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>38</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="66" t="s">
-        <v>73</v>
+      <c r="G9" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>41</v>
-      </c>
       <c r="J9" s="65" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>14</v>
+      <c r="G10" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J10" s="65" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>14</v>
+      <c r="G11" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J11" s="65" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="8" t="s">
-        <v>14</v>
+      <c r="G12" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J12" s="65" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>14</v>
+      <c r="G13" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J13" s="65" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>10</v>
@@ -1884,7 +1884,7 @@
         <v>11</v>
       </c>
       <c r="D14" s="61" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>11</v>
@@ -1893,243 +1893,243 @@
         <v>13</v>
       </c>
       <c r="G14" s="68" t="s">
-        <v>143</v>
+        <v>72</v>
       </c>
       <c r="H14" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="11" t="s">
         <v>15</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>16</v>
       </c>
       <c r="J14" s="16"/>
     </row>
     <row r="15" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>56</v>
-      </c>
       <c r="E15" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="14" t="s">
-        <v>14</v>
+      <c r="G15" s="68" t="s">
+        <v>72</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I15" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="J15" s="16" t="s">
         <v>57</v>
-      </c>
-      <c r="J15" s="16" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>60</v>
-      </c>
       <c r="E16" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="14" t="s">
-        <v>14</v>
+      <c r="G16" s="68" t="s">
+        <v>72</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I16" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="J16" s="16" t="s">
         <v>61</v>
-      </c>
-      <c r="J16" s="16" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>64</v>
-      </c>
       <c r="E17" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="14" t="s">
-        <v>14</v>
+      <c r="G17" s="68" t="s">
+        <v>72</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>67</v>
-      </c>
       <c r="E18" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="14" t="s">
-        <v>14</v>
+      <c r="G18" s="68" t="s">
+        <v>72</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I18" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="J18" s="16" t="s">
         <v>68</v>
-      </c>
-      <c r="J18" s="16" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>72</v>
-      </c>
       <c r="E19" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="8" t="s">
-        <v>73</v>
+      <c r="G19" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H19" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I19" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>41</v>
-      </c>
       <c r="J19" s="65" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>75</v>
-      </c>
       <c r="E20" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="8" t="s">
-        <v>14</v>
+      <c r="G20" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J20" s="65" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>77</v>
-      </c>
       <c r="E21" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="8" t="s">
-        <v>14</v>
+      <c r="G21" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J21" s="65" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>10</v>
@@ -2138,220 +2138,220 @@
         <v>11</v>
       </c>
       <c r="D22" s="62" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="G22" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="H22" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="G22" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="17" t="s">
+      <c r="I22" s="17" t="s">
         <v>82</v>
-      </c>
-      <c r="I22" s="17" t="s">
-        <v>83</v>
       </c>
       <c r="J22" s="22"/>
     </row>
     <row r="23" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" s="22" t="s">
+      <c r="E23" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="G23" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="E23" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="G23" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H23" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="I23" s="20" t="s">
+      <c r="J23" s="22" t="s">
         <v>86</v>
-      </c>
-      <c r="J23" s="22" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="B24" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="22" t="s">
+      <c r="E24" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="G24" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="E24" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="G24" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H24" s="20" t="s">
+      <c r="I24" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="I24" s="20" t="s">
+      <c r="J24" s="22" t="s">
         <v>91</v>
-      </c>
-      <c r="J24" s="22" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="22" t="s">
+      <c r="E25" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="22" t="s">
+      <c r="G25" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="E25" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="G25" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H25" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="I25" s="20" t="s">
+      <c r="J25" s="22" t="s">
         <v>95</v>
-      </c>
-      <c r="J25" s="22" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" s="22" t="s">
+      <c r="E26" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="G26" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="E26" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="F26" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="G26" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H26" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="I26" s="20" t="s">
+      <c r="J26" s="22" t="s">
         <v>99</v>
-      </c>
-      <c r="J26" s="22" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C27" s="10" t="s">
+      <c r="E27" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="G27" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E27" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>103</v>
-      </c>
       <c r="J27" s="65" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="10" t="s">
+      <c r="E28" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F28" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="G28" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I28" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="E28" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>106</v>
-      </c>
       <c r="J28" s="65" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B29" s="24" t="s">
         <v>10</v>
@@ -2360,247 +2360,247 @@
         <v>11</v>
       </c>
       <c r="D29" s="63" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E29" s="23" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" s="77" t="s">
+        <v>72</v>
+      </c>
+      <c r="H29" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="G29" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="H29" s="23" t="s">
+      <c r="I29" s="23" t="s">
         <v>110</v>
-      </c>
-      <c r="I29" s="23" t="s">
-        <v>111</v>
       </c>
       <c r="J29" s="25"/>
     </row>
     <row r="30" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="D30" s="28" t="s">
+      <c r="E30" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="G30" s="77" t="s">
+        <v>72</v>
+      </c>
+      <c r="H30" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="J30" s="28" t="s">
         <v>113</v>
-      </c>
-      <c r="E30" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="G30" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="H30" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="I30" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="J30" s="28" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="B31" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="D31" s="28" t="s">
+      <c r="E31" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="G31" s="77" t="s">
+        <v>72</v>
+      </c>
+      <c r="H31" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="I31" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="J31" s="28" t="s">
         <v>116</v>
-      </c>
-      <c r="E31" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="G31" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="I31" s="26" t="s">
-        <v>99</v>
-      </c>
-      <c r="J31" s="28" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="B32" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C32" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="D32" s="28" t="s">
+      <c r="E32" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="G32" s="77" t="s">
+        <v>72</v>
+      </c>
+      <c r="H32" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="I32" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="E32" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="G32" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="H32" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="I32" s="26" t="s">
+      <c r="J32" s="28" t="s">
         <v>120</v>
-      </c>
-      <c r="J32" s="28" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D33" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="D33" s="28" t="s">
+      <c r="E33" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="G33" s="77" t="s">
+        <v>72</v>
+      </c>
+      <c r="H33" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="I33" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="J33" s="28" t="s">
         <v>123</v>
-      </c>
-      <c r="E33" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="F33" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="H33" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="I33" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="J33" s="28" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="57" t="s">
+        <v>124</v>
+      </c>
+      <c r="B34" s="57" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="58" t="s">
         <v>125</v>
       </c>
-      <c r="B34" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="58" t="s">
-        <v>108</v>
-      </c>
-      <c r="D34" s="58" t="s">
-        <v>126</v>
-      </c>
       <c r="E34" s="57" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="G34" s="57" t="s">
-        <v>14</v>
+      <c r="G34" s="75" t="s">
+        <v>72</v>
       </c>
       <c r="H34" s="57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I34" s="57" t="s">
+        <v>126</v>
+      </c>
+      <c r="J34" s="65" t="s">
         <v>127</v>
-      </c>
-      <c r="J34" s="65" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="66" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D35" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G35" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I35" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="E35" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>134</v>
-      </c>
       <c r="J35" s="65" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="66" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D36" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G36" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I36" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G36" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I36" s="8" t="s">
-        <v>131</v>
-      </c>
       <c r="J36" s="65" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2628,7 +2628,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2641,16 +2641,16 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
@@ -2661,39 +2661,39 @@
         <v>13</v>
       </c>
       <c r="B3" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="59" t="s">
         <v>140</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="D3" s="59" t="s">
+        <v>188</v>
+      </c>
+      <c r="E3" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="59" t="s">
-        <v>192</v>
-      </c>
-      <c r="E3" s="59" t="s">
+      <c r="F3" s="30" t="s">
         <v>142</v>
-      </c>
-      <c r="F3" s="30" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="D4" s="69" t="s">
         <v>145</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="E4" s="69" t="s">
         <v>146</v>
       </c>
-      <c r="E4" s="69" t="s">
+      <c r="F4" s="33" t="s">
         <v>147</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2719,7 +2719,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2729,22 +2729,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
@@ -2758,10 +2758,10 @@
         <v>13</v>
       </c>
       <c r="D3" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="E3" s="31" t="s">
         <v>155</v>
-      </c>
-      <c r="E3" s="31" t="s">
-        <v>156</v>
       </c>
       <c r="F3" s="30">
         <f>9+7</f>
@@ -2770,19 +2770,19 @@
     </row>
     <row r="4" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>53</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>54</v>
       </c>
       <c r="C4" s="36" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="37" t="s">
         <v>157</v>
-      </c>
-      <c r="E4" s="37" t="s">
-        <v>158</v>
       </c>
       <c r="F4" s="36">
         <f>10+5</f>
@@ -2791,19 +2791,19 @@
     </row>
     <row r="5" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="C5" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="33" t="s">
-        <v>81</v>
-      </c>
       <c r="D5" s="34" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" s="34" t="s">
         <v>159</v>
-      </c>
-      <c r="E5" s="34" t="s">
-        <v>160</v>
       </c>
       <c r="F5" s="33">
         <f>13+2</f>
@@ -2812,19 +2812,19 @@
     </row>
     <row r="6" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="C6" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="C6" s="39" t="s">
-        <v>109</v>
-      </c>
       <c r="D6" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6" s="40" t="s">
         <v>161</v>
-      </c>
-      <c r="E6" s="40" t="s">
-        <v>162</v>
       </c>
       <c r="F6" s="39">
         <f>9+3</f>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E7" s="41" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F7" s="41">
         <f>SUM(F3:F6)</f>
@@ -2864,7 +2864,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="72" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -2876,25 +2876,25 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>7</v>
@@ -2902,138 +2902,136 @@
     </row>
     <row r="3" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="42" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" s="43" t="s">
         <v>170</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="C3" s="44" t="s">
         <v>171</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="D3" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="D3" s="44" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="44" t="s">
+      <c r="G3" s="43" t="s">
         <v>173</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="H3" s="44" t="s">
         <v>174</v>
-      </c>
-      <c r="H3" s="44" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="45" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="C4" s="47" t="s">
         <v>177</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="D4" s="47" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="47" t="s">
+        <v>172</v>
+      </c>
+      <c r="G4" s="46" t="s">
         <v>178</v>
       </c>
-      <c r="D4" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="E4" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="47" t="s">
-        <v>173</v>
-      </c>
-      <c r="G4" s="46" t="s">
-        <v>179</v>
-      </c>
       <c r="H4" s="47" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="48" t="s">
+        <v>179</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>209</v>
+      </c>
+      <c r="C5" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>208</v>
+      </c>
+      <c r="E5" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="49" t="s">
-        <v>181</v>
-      </c>
-      <c r="C5" s="50" t="s">
-        <v>172</v>
-      </c>
-      <c r="D5" s="50" t="s">
-        <v>212</v>
-      </c>
-      <c r="E5" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="49" t="s">
-        <v>182</v>
-      </c>
       <c r="H5" s="50" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>182</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" s="53" t="s">
+        <v>208</v>
+      </c>
+      <c r="E6" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="52" t="s">
         <v>183</v>
       </c>
-      <c r="B6" s="52" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>172</v>
-      </c>
-      <c r="D6" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="E6" s="53" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="53" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="52" t="s">
-        <v>185</v>
-      </c>
       <c r="H6" s="53" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="54" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="55" t="s">
+        <v>185</v>
+      </c>
+      <c r="C7" s="56" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="D7" s="56" t="s">
+        <v>208</v>
+      </c>
+      <c r="E7" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="56" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="55" t="s">
         <v>187</v>
       </c>
-      <c r="C7" s="56" t="s">
-        <v>188</v>
-      </c>
-      <c r="D7" s="56" t="s">
-        <v>212</v>
-      </c>
-      <c r="E7" s="56" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="56" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="55" t="s">
-        <v>189</v>
-      </c>
       <c r="H7" s="56" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="74" t="s">
-        <v>190</v>
-      </c>
+      <c r="A8" s="74"/>
       <c r="B8" s="73"/>
       <c r="C8" s="73"/>
       <c r="D8" s="73"/>
@@ -3043,9 +3041,7 @@
       <c r="H8" s="73"/>
     </row>
     <row r="9" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="74" t="s">
-        <v>191</v>
-      </c>
+      <c r="A9" s="74"/>
       <c r="B9" s="73"/>
       <c r="C9" s="73"/>
       <c r="D9" s="73"/>

</xml_diff>